<commit_message>
revised filtering and extraction functions
</commit_message>
<xml_diff>
--- a/www/marker_info2.xlsx
+++ b/www/marker_info2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ketchup\Desktop\restful-forensics-shinyapp\www\sample_files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lcbsa\OneDrive\Desktop\restful-forensics v2\www\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E75F46E-6D3B-49D9-9508-48B3441E000E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6B3021D-B3DB-4B18-B7CD-E126C1A5E416}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9012" yWindow="756" windowWidth="13968" windowHeight="12024" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5304" yWindow="1332" windowWidth="7800" windowHeight="8928" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>rs2139931</t>
   </si>
@@ -46,13 +46,19 @@
   </si>
   <si>
     <t>rs7531501</t>
+  </si>
+  <si>
+    <t>rs6054465</t>
+  </si>
+  <si>
+    <t>rs310644</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -71,6 +77,20 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -154,7 +174,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -171,6 +191,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -451,7 +473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.6640625" customWidth="1"/>
@@ -501,7 +523,7 @@
         <v>1249187</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
@@ -510,6 +532,28 @@
       </c>
       <c r="C5" s="5">
         <v>234338303</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="6">
+        <v>20</v>
+      </c>
+      <c r="C6" s="6">
+        <v>6673018</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="6">
+        <v>20</v>
+      </c>
+      <c r="C7" s="7">
+        <v>62159504</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
made rsid optional in pos file functions
</commit_message>
<xml_diff>
--- a/www/marker_info2.xlsx
+++ b/www/marker_info2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lcbsa\OneDrive\Desktop\restful-forensics v2\www\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6B3021D-B3DB-4B18-B7CD-E126C1A5E416}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F2BBDEC-6D72-4C18-B3D3-4F35DA1648D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5304" yWindow="1332" windowWidth="7800" windowHeight="8928" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2595" yWindow="2385" windowWidth="13635" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,10 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
-  <si>
-    <t>rs2139931</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>chr</t>
   </si>
@@ -39,49 +36,28 @@
     <t>pos</t>
   </si>
   <si>
-    <t>rs2814778</t>
-  </si>
-  <si>
-    <t>rs12142199</t>
-  </si>
-  <si>
-    <t>rs7531501</t>
-  </si>
-  <si>
-    <t>rs6054465</t>
-  </si>
-  <si>
-    <t>rs310644</t>
+    <t>rs4411548</t>
+  </si>
+  <si>
+    <t>rs2593595</t>
+  </si>
+  <si>
+    <t>rs17642714</t>
+  </si>
+  <si>
+    <t>rs4471745</t>
+  </si>
+  <si>
+    <t>rs11652805</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -102,27 +78,12 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -140,59 +101,19 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="medium">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -473,87 +394,77 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.6640625" customWidth="1"/>
+    <col min="1" max="1" width="11.7109375" customWidth="1"/>
+    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+    </row>
+    <row r="2" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="2">
-        <v>1</v>
+      <c r="B2" s="1">
+        <v>17</v>
       </c>
       <c r="C2" s="2">
-        <v>84590527</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+        <v>42506515</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="4">
-        <v>1</v>
-      </c>
-      <c r="C3" s="4">
-        <v>159174683</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
+      <c r="B3" s="1">
+        <v>17</v>
+      </c>
+      <c r="C3" s="2">
+        <v>41056245</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="5">
-        <v>1</v>
-      </c>
-      <c r="C4" s="5">
-        <v>1249187</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
+      <c r="B4" s="1">
+        <v>17</v>
+      </c>
+      <c r="C4" s="2">
+        <v>48726132</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="5">
-        <v>1</v>
-      </c>
-      <c r="C5" s="5">
-        <v>234338303</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="6" t="s">
+      <c r="B5" s="1">
+        <v>17</v>
+      </c>
+      <c r="C5" s="2">
+        <v>55491523</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="6">
-        <v>20</v>
-      </c>
-      <c r="C6" s="6">
-        <v>6673018</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" s="6">
-        <v>20</v>
-      </c>
-      <c r="C7" s="7">
-        <v>62159504</v>
+      <c r="B6" s="1">
+        <v>17</v>
+      </c>
+      <c r="C6" s="2">
+        <v>62987151</v>
       </c>
     </row>
   </sheetData>

</xml_diff>